<commit_message>
Sync P006 and P005 Excel review sheets with illustrated-mechanism hyperlinks
</commit_message>
<xml_diff>
--- a/papers/P005/P005_工程复现问题清单_v1.xlsx
+++ b/papers/P005/P005_工程复现问题清单_v1.xlsx
@@ -30,13 +30,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF142B46"/>
+        <fgColor rgb="FF122C45"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F5F9"/>
+        <fgColor rgb="FFF0F5FA"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -55,13 +55,13 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment wrapText="1" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment wrapText="1" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment wrapText="1" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -75,12 +75,12 @@
   <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="25"/>
   <cols>
-    <col min="1" max="1" width="26" customWidth="1"/>
-    <col min="2" max="2" width="53" customWidth="1"/>
-    <col min="3" max="3" width="92" customWidth="1"/>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="2" width="52" customWidth="1"/>
+    <col min="3" max="3" width="94" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1">
+    <row r="1" ht="35" customHeight="1">
       <c r="A1" t="inlineStr" s="1">
         <is>
           <t xml:space="preserve">主题</t>
@@ -97,7 +97,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="94" customHeight="1">
+    <row r="2" ht="88" customHeight="1">
       <c r="A2" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">市场环境究竟是什么？</t>
@@ -114,7 +114,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="94" customHeight="1">
+    <row r="3" ht="88" customHeight="1">
       <c r="A3" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">LLM底座与职责</t>
@@ -131,7 +131,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="94" customHeight="1">
+    <row r="4" ht="100" customHeight="1">
       <c r="A4" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">市场信息怎样与因子池结合？</t>
@@ -148,7 +148,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="94" customHeight="1">
+    <row r="5" ht="88" customHeight="1">
       <c r="A5" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">当前因子池指什么？</t>
@@ -165,7 +165,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="94" customHeight="1">
+    <row r="6" ht="88" customHeight="1">
       <c r="A6" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">初始任务与因子生成形式</t>
@@ -182,7 +182,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="94" customHeight="1">
+    <row r="7" ht="88" customHeight="1">
       <c r="A7" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">池级边际贡献的计算单位</t>
@@ -199,7 +199,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="94" customHeight="1">
+    <row r="8" ht="124" customHeight="1">
       <c r="A8" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">整个池怎么得到分数？</t>
@@ -212,11 +212,11 @@
       </c>
       <c r="C8" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">先用近期约126个交易日的历史数据，对池内因子截面Rank信号拟合非负岭回归式组合权重，汇总成Meta-alpha，再算组合IC、RankIC及多样性/稳定性等池指标。新因子可能与现有因子重复，单项IC虽高却不改善组合，因此边际池收益≤0会被拒绝。</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="94" customHeight="1">
+          <t xml:space="preserve">先用近期约126个交易日的数据，通过“非负岭回归”给池内各因子拟合组合权重：权重不能小于零，太大的权重还会受到惩罚。把因子按权重相加成Meta-alpha，再算整池IC、RankIC和多样性/稳定性得分。新因子单独IC好却与旧因子重复，也可能不增加整池价值。用数字和图讲清楚：https://github.com/epshoron/JXwork/blob/main/papers/P005/P005_NONNEGATIVE_RIDGE_GUIDE.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="88" customHeight="1">
       <c r="A9" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">质量检查与评分层次</t>
@@ -233,7 +233,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="94" customHeight="1">
+    <row r="10" ht="100" customHeight="1">
       <c r="A10" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">池状态具体怎样更新？</t>
@@ -250,7 +250,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="94" customHeight="1">
+    <row r="11" ht="88" customHeight="1">
       <c r="A11" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">多轮反馈怎么闭环？</t>
@@ -267,7 +267,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="94" customHeight="1">
+    <row r="12" ht="100" customHeight="1">
       <c r="A12" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">调度与优化对象</t>
@@ -284,7 +284,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="108" customHeight="1">
+    <row r="13" ht="112" customHeight="1">
       <c r="A13" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">GRPO本质是什么？</t>
@@ -301,7 +301,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="94" customHeight="1">
+    <row r="14" ht="88" customHeight="1">
       <c r="A14" t="inlineStr" s="0">
         <is>
           <t xml:space="preserve">训练和实际使用怎样区分？</t>
@@ -318,7 +318,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="82" customHeight="1">
+    <row r="15" ht="88" customHeight="1">
       <c r="A15" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">公开实现与复现边界</t>
@@ -337,5 +337,8 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:C15"/>
+  <hyperlinks>
+    <hyperlink ref="C8" r:id="rId1" tooltip="查看详细机制图解"/>
+  </hyperlinks>
 </worksheet>
 </file>
</xml_diff>